<commit_message>
subidos primeros consorcios en primer etapa de septiembre
</commit_message>
<xml_diff>
--- a/DRAGO/Octubre/EXPENSAS-Octubre.xlsx
+++ b/DRAGO/Octubre/EXPENSAS-Octubre.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\RC CONSORCIO 2025\DRAGO\Octubre\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\DRAGO\Octubre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A7D5AE-8C89-4D8B-8D7B-FD13FC5521E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F56F355F-0E5C-4C33-8D36-2A9F4C99B9CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="detalle y gastos" sheetId="3" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="98">
   <si>
     <t>UF</t>
   </si>
@@ -193,9 +193,6 @@
     <t xml:space="preserve">Seguro Integral </t>
   </si>
   <si>
-    <t>DEUDAS</t>
-  </si>
-  <si>
     <t>Liquidación de mes: JULIO 2022</t>
   </si>
   <si>
@@ -226,9 +223,6 @@
     <t>Enzo</t>
   </si>
   <si>
-    <t>Liquidación de mes: DICIEMBRE 2023</t>
-  </si>
-  <si>
     <t>CAJA EXTRAORDINARIA</t>
   </si>
   <si>
@@ -241,15 +235,6 @@
     <t>Sueldo Sra. Monica</t>
   </si>
   <si>
-    <t>ENERO</t>
-  </si>
-  <si>
-    <t>PUNITORIOS DE 5 MESES</t>
-  </si>
-  <si>
-    <t>EXTRAORD</t>
-  </si>
-  <si>
     <t>Honorarios administracion</t>
   </si>
   <si>
@@ -323,6 +308,18 @@
   </si>
   <si>
     <t>Estefania</t>
+  </si>
+  <si>
+    <t>Expensas extraordinarias jun 2024</t>
+  </si>
+  <si>
+    <t>Expensas extr.</t>
+  </si>
+  <si>
+    <t>Intereses (3% c/ mes)</t>
+  </si>
+  <si>
+    <t>Liquidación de mes</t>
   </si>
 </sst>
 </file>
@@ -717,20 +714,7 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -741,28 +725,6 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -876,6 +838,51 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -887,7 +894,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -941,7 +948,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
@@ -966,7 +972,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="1" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -980,33 +985,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="11" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1019,12 +1004,6 @@
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1043,32 +1022,32 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="3" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="1" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="3" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="1" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="26" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1076,65 +1055,91 @@
     </xf>
     <xf numFmtId="3" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="4" fontId="16" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="16" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1503,60 +1508,60 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:H58"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="40.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="25"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>39</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1564,7 +1569,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -1572,217 +1577,217 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="23" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="86" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="77"/>
-      <c r="C16" s="119"/>
-    </row>
-    <row r="17" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="77" t="s">
+      <c r="B16" s="65"/>
+      <c r="C16" s="105"/>
+    </row>
+    <row r="17" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="65" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="87" t="s">
-        <v>85</v>
-      </c>
-      <c r="C17" s="138">
+      <c r="B17" s="73" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="108">
         <v>41718</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="14"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="77" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="88"/>
-      <c r="C18" s="138">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="65" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="74"/>
+      <c r="C18" s="108">
         <v>4519.75</v>
       </c>
-      <c r="D18" s="49"/>
+      <c r="D18" s="47"/>
       <c r="E18" s="14"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="77" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="89" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" s="138">
+      <c r="B19" s="75" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="108">
         <v>16346.58</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="14"/>
       <c r="F19" s="18"/>
-      <c r="H19" s="121"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="77" t="s">
+      <c r="H19" s="107"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="89" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="139">
+      <c r="B20" s="75" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="109">
         <v>168796.55</v>
       </c>
-      <c r="D20" s="49"/>
+      <c r="D20" s="47"/>
       <c r="F20" s="14"/>
-      <c r="H20" s="121"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="77" t="s">
+      <c r="H20" s="107"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="89" t="s">
-        <v>74</v>
-      </c>
-      <c r="C21" s="138">
+      <c r="B21" s="75" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="108">
         <v>53465</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="14"/>
       <c r="H21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="90"/>
-      <c r="B22" s="91"/>
-      <c r="C22" s="64">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="76"/>
+      <c r="B22" s="77"/>
+      <c r="C22" s="58">
         <f>SUM(C17:C21)</f>
         <v>284845.88</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="86" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="89"/>
-      <c r="C23" s="119"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="77" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="92" t="s">
-        <v>90</v>
-      </c>
-      <c r="C24" s="138">
+      <c r="B23" s="75"/>
+      <c r="C23" s="105"/>
+    </row>
+    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="65" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24" s="78" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" s="108">
         <f>68460+68460*5%</f>
         <v>71883</v>
       </c>
       <c r="F24" s="22"/>
     </row>
-    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="77" t="s">
-        <v>96</v>
-      </c>
-      <c r="B25" s="92"/>
-      <c r="C25" s="138">
+    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="65" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="78"/>
+      <c r="C25" s="108">
         <v>60899.97</v>
       </c>
       <c r="F25" s="22"/>
     </row>
-    <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="77" t="s">
-        <v>94</v>
-      </c>
-      <c r="B26" s="92"/>
-      <c r="C26" s="138">
+    <row r="26" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="78"/>
+      <c r="C26" s="108">
         <v>15000</v>
       </c>
       <c r="F26" s="22"/>
     </row>
-    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="77" t="s">
-        <v>88</v>
-      </c>
-      <c r="B27" s="92"/>
-      <c r="C27" s="84"/>
+    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="78"/>
+      <c r="C27" s="70"/>
       <c r="F27" s="22"/>
     </row>
-    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="77" t="s">
-        <v>80</v>
-      </c>
-      <c r="B28" s="89"/>
-      <c r="C28" s="85"/>
+    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="65" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="75"/>
+      <c r="C28" s="71"/>
       <c r="D28" s="5"/>
       <c r="E28" s="14"/>
       <c r="F28" s="22"/>
     </row>
-    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="90"/>
-      <c r="B29" s="91"/>
-      <c r="C29" s="64">
+    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="76"/>
+      <c r="B29" s="77"/>
+      <c r="C29" s="58">
         <f>SUM(C23:C28)</f>
         <v>147782.97</v>
       </c>
       <c r="F29" s="22"/>
     </row>
-    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="80" t="s">
-        <v>79</v>
-      </c>
-      <c r="B30" s="80"/>
-      <c r="C30" s="93">
+    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="68" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" s="68"/>
+      <c r="C30" s="79">
         <f>+C29+C22</f>
         <v>432628.85</v>
       </c>
       <c r="F30" s="22"/>
     </row>
-    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C31" s="65"/>
+    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C31" s="59"/>
       <c r="F31" s="22"/>
     </row>
-    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C32" s="65"/>
+      <c r="C32" s="59"/>
       <c r="F32" s="22"/>
     </row>
-    <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="140" t="s">
-        <v>92</v>
-      </c>
-      <c r="B33" s="141"/>
-      <c r="C33" s="142">
+    <row r="33" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="111" t="s">
+        <v>87</v>
+      </c>
+      <c r="B33" s="112"/>
+      <c r="C33" s="110">
         <f>68000+40000</f>
         <v>108000</v>
       </c>
       <c r="F33" s="22"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="77"/>
-      <c r="B34" s="77"/>
-      <c r="C34" s="85"/>
+    <row r="34" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="65"/>
+      <c r="B34" s="65"/>
+      <c r="C34" s="71"/>
       <c r="F34" s="22"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="77"/>
-      <c r="B35" s="77"/>
-      <c r="C35" s="85"/>
+    <row r="35" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="65"/>
+      <c r="B35" s="65"/>
+      <c r="C35" s="71"/>
       <c r="F35" s="22"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C36" s="67"/>
+    <row r="36" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C36" s="60"/>
       <c r="F36" s="22"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="23" t="s">
         <v>43</v>
       </c>
@@ -1793,148 +1798,148 @@
       </c>
       <c r="E37" s="14"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="35" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="35"/>
-      <c r="C39" s="36">
+      <c r="B39" s="34"/>
+      <c r="C39" s="35">
         <f>+C37+C30</f>
         <v>540628.85</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="37" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="34"/>
-      <c r="C42" s="41">
+      <c r="B42" s="33"/>
+      <c r="C42" s="40">
         <v>283181.4519533891</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>9</v>
       </c>
-      <c r="C43" s="33">
+      <c r="C43" s="32">
         <f>'prorrateo '!F13</f>
         <v>360987.84211000003</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>77</v>
-      </c>
-      <c r="C44" s="94"/>
+        <v>72</v>
+      </c>
+      <c r="C44" s="80"/>
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>93</v>
-      </c>
-      <c r="C45" s="94">
+        <v>88</v>
+      </c>
+      <c r="C45" s="80">
         <v>-20000</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" s="94">
+        <v>90</v>
+      </c>
+      <c r="C46" s="80">
         <f>-C37</f>
         <v>-108000</v>
       </c>
       <c r="D46" s="14"/>
       <c r="E46" s="14"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>76</v>
-      </c>
-      <c r="C47" s="94">
+        <v>71</v>
+      </c>
+      <c r="C47" s="80">
         <f>-(C30-C28)</f>
         <v>-432628.85</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="37" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="B48" s="34"/>
-      <c r="C48" s="41">
+      <c r="B48" s="33"/>
+      <c r="C48" s="40">
         <f>SUM(C42:C47)</f>
         <v>83540.444063389092</v>
       </c>
       <c r="D48" s="6"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="19"/>
       <c r="B49" s="18"/>
       <c r="C49" s="20"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="19"/>
       <c r="B50" s="18"/>
       <c r="C50" s="20"/>
-      <c r="F50" s="95"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F50" s="81"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="19"/>
       <c r="B51" s="18"/>
       <c r="C51" s="20"/>
     </row>
-    <row r="52" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="76" t="s">
-        <v>67</v>
-      </c>
-      <c r="B52" s="99"/>
-      <c r="C52" s="100">
+    <row r="52" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A52" s="64" t="s">
+        <v>65</v>
+      </c>
+      <c r="B52" s="85"/>
+      <c r="C52" s="86">
         <v>109834.99657000002</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="77"/>
-      <c r="B53" s="77"/>
-      <c r="C53" s="83"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="80" t="s">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="65"/>
+      <c r="B53" s="65"/>
+      <c r="C53" s="69"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="78"/>
-      <c r="C54" s="79">
+      <c r="B54" s="66"/>
+      <c r="C54" s="67">
         <f>SUM(C52:C53)</f>
         <v>109834.99657000002</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="18"/>
       <c r="B55" s="18"/>
       <c r="C55" s="18"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="18"/>
       <c r="B56" s="18"/>
       <c r="C56" s="18"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="18"/>
       <c r="B57" s="18"/>
       <c r="C57" s="18"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="18"/>
       <c r="B58" s="18"/>
       <c r="C58" s="18"/>
@@ -1959,28 +1964,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="8" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" hidden="1" customWidth="1"/>
-    <col min="11" max="12" width="12.42578125" customWidth="1"/>
-    <col min="13" max="13" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="21"/>
+    <col min="3" max="3" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="10.5546875" hidden="1" customWidth="1"/>
+    <col min="11" max="12" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="51">
+      <c r="E1" s="49">
         <v>396674.61</v>
       </c>
       <c r="G1" t="str">
@@ -1988,494 +1993,494 @@
         <v>Vto. 14/11</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="106" t="str">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="92" t="str">
         <f>'detalle y gastos'!B7</f>
         <v>LIQUIDACIÓN EXPENSAS OCTUBRE 2025</v>
       </c>
-      <c r="B2" s="101"/>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="108" t="s">
+      <c r="B2" s="87"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="94" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="102"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="124"/>
-      <c r="B3" s="122" t="s">
+      <c r="F2" s="87"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="87"/>
+      <c r="L2" s="87"/>
+      <c r="M2" s="88"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="115"/>
+      <c r="B3" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="130" t="s">
+      <c r="C3" s="121" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="131" t="s">
-        <v>60</v>
-      </c>
-      <c r="E3" s="122" t="s">
+      <c r="D3" s="122" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="113" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="128" t="s">
+      <c r="F3" s="119" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="130" t="s">
-        <v>58</v>
-      </c>
-      <c r="H3" s="128" t="s">
+      <c r="G3" s="121" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="119" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="130" t="s">
+      <c r="I3" s="121" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="132" t="s">
+      <c r="J3" s="123" t="s">
+        <v>73</v>
+      </c>
+      <c r="K3" s="117" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="117" t="s">
+        <v>77</v>
+      </c>
+      <c r="M3" s="117" t="s">
         <v>78</v>
       </c>
-      <c r="K3" s="126" t="s">
-        <v>81</v>
-      </c>
-      <c r="L3" s="126" t="s">
-        <v>82</v>
-      </c>
-      <c r="M3" s="126" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="125"/>
-      <c r="B4" s="123"/>
-      <c r="C4" s="130"/>
-      <c r="D4" s="131"/>
-      <c r="E4" s="123"/>
-      <c r="F4" s="129"/>
-      <c r="G4" s="130"/>
-      <c r="H4" s="129"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="132"/>
-      <c r="K4" s="127"/>
-      <c r="L4" s="127"/>
-      <c r="M4" s="127"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="103">
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="116"/>
+      <c r="B4" s="114"/>
+      <c r="C4" s="121"/>
+      <c r="D4" s="122"/>
+      <c r="E4" s="114"/>
+      <c r="F4" s="120"/>
+      <c r="G4" s="121"/>
+      <c r="H4" s="120"/>
+      <c r="I4" s="121"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="118"/>
+      <c r="L4" s="118"/>
+      <c r="M4" s="118"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="89">
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="62" t="s">
+      <c r="C5" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="47">
+      <c r="D5" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="46">
         <v>47997.627809999998</v>
       </c>
-      <c r="F5" s="120">
+      <c r="F5" s="106">
         <f t="shared" ref="F5:F11" si="0">E5</f>
         <v>47997.627809999998</v>
       </c>
-      <c r="G5" s="47">
+      <c r="G5" s="46">
         <f>E5-F5</f>
         <v>0</v>
       </c>
-      <c r="H5" s="47">
+      <c r="H5" s="46">
         <f>IF(G5&gt;0,G5*5%,0)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="109">
+      <c r="I5" s="95">
         <v>0.121</v>
       </c>
-      <c r="J5" s="98"/>
-      <c r="K5" s="110">
+      <c r="J5" s="84"/>
+      <c r="K5" s="96">
         <f>E1*I5</f>
         <v>47997.627809999998</v>
       </c>
-      <c r="L5" s="110">
+      <c r="L5" s="96">
         <f>E5-F5+H5+K5+J5</f>
         <v>47997.627809999998</v>
       </c>
-      <c r="M5" s="111">
+      <c r="M5" s="97">
         <f>L5+L5*4%</f>
         <v>49917.532922400002</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="103">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="89">
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="62" t="s">
+      <c r="C6" s="57" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="62" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="47">
+      <c r="D6" s="57" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="46">
         <v>48394.30242</v>
       </c>
-      <c r="F6" s="120">
+      <c r="F6" s="106">
         <f t="shared" si="0"/>
         <v>48394.30242</v>
       </c>
-      <c r="G6" s="47">
+      <c r="G6" s="46">
         <f t="shared" ref="G6:G12" si="1">E6-F6</f>
         <v>0</v>
       </c>
-      <c r="H6" s="47">
+      <c r="H6" s="46">
         <f t="shared" ref="H6:H12" si="2">IF(G6&gt;0,G6*5%,0)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="109">
+      <c r="I6" s="95">
         <v>0.122</v>
       </c>
-      <c r="J6" s="98"/>
-      <c r="K6" s="110">
+      <c r="J6" s="84"/>
+      <c r="K6" s="96">
         <f>E1*I6</f>
         <v>48394.30242</v>
       </c>
-      <c r="L6" s="110">
+      <c r="L6" s="96">
         <f t="shared" ref="L6:L12" si="3">E6-F6+H6+K6+J6</f>
         <v>48394.30242</v>
       </c>
-      <c r="M6" s="111">
+      <c r="M6" s="97">
         <f t="shared" ref="M6:M12" si="4">L6+L6*4%</f>
         <v>50330.074516799999</v>
       </c>
-      <c r="O6" s="118"/>
-      <c r="Q6" s="117"/>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="103">
+      <c r="O6" s="104"/>
+      <c r="Q6" s="103"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="89">
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="62" t="s">
+      <c r="C7" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="62" t="s">
-        <v>84</v>
-      </c>
-      <c r="E7" s="47">
+      <c r="D7" s="57" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" s="46">
         <v>46410.929369999998</v>
       </c>
-      <c r="F7" s="120">
+      <c r="F7" s="106">
         <f>E7</f>
         <v>46410.929369999998</v>
       </c>
-      <c r="G7" s="47">
+      <c r="G7" s="46">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H7" s="47">
+      <c r="H7" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I7" s="109">
+      <c r="I7" s="95">
         <v>0.11700000000000001</v>
       </c>
-      <c r="J7" s="98"/>
-      <c r="K7" s="110">
+      <c r="J7" s="84"/>
+      <c r="K7" s="96">
         <f>E1*I7</f>
         <v>46410.929369999998</v>
       </c>
-      <c r="L7" s="110">
+      <c r="L7" s="96">
         <f t="shared" si="3"/>
         <v>46410.929369999998</v>
       </c>
-      <c r="M7" s="111">
+      <c r="M7" s="97">
         <f t="shared" si="4"/>
         <v>48267.366544799996</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="103">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="89">
         <v>4</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="62" t="s">
+      <c r="C8" s="57" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="62" t="s">
-        <v>87</v>
-      </c>
-      <c r="E8" s="120">
+      <c r="D8" s="57" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="106">
         <v>46410.929369999998</v>
       </c>
-      <c r="F8" s="120">
+      <c r="F8" s="106">
         <v>63085.21</v>
       </c>
-      <c r="G8" s="47">
+      <c r="G8" s="46">
         <f t="shared" si="1"/>
         <v>-16674.280630000001</v>
       </c>
-      <c r="H8" s="47">
+      <c r="H8" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I8" s="109">
+      <c r="I8" s="95">
         <v>0.11700000000000001</v>
       </c>
-      <c r="J8" s="98"/>
-      <c r="K8" s="110">
+      <c r="J8" s="84"/>
+      <c r="K8" s="96">
         <f>E1*I8</f>
         <v>46410.929369999998</v>
       </c>
-      <c r="L8" s="110">
+      <c r="L8" s="96">
         <f t="shared" si="3"/>
         <v>29736.648739999997</v>
       </c>
-      <c r="M8" s="111">
+      <c r="M8" s="97">
         <f t="shared" si="4"/>
         <v>30926.114689599995</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="103">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="89">
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="62" t="s">
+      <c r="C9" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="62" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" s="47">
+      <c r="D9" s="57" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="46">
         <v>54344.421570000006</v>
       </c>
-      <c r="F9" s="120">
+      <c r="F9" s="106">
         <f>E9</f>
         <v>54344.421570000006</v>
       </c>
-      <c r="G9" s="47">
+      <c r="G9" s="46">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H9" s="47">
+      <c r="H9" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I9" s="109">
+      <c r="I9" s="95">
         <v>0.13700000000000001</v>
       </c>
-      <c r="J9" s="98"/>
-      <c r="K9" s="110">
+      <c r="J9" s="84"/>
+      <c r="K9" s="96">
         <f>E1*I9</f>
         <v>54344.421570000006</v>
       </c>
-      <c r="L9" s="110">
+      <c r="L9" s="96">
         <f t="shared" si="3"/>
         <v>54344.421570000006</v>
       </c>
-      <c r="M9" s="111">
+      <c r="M9" s="97">
         <f t="shared" si="4"/>
         <v>56518.198432800004</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="103">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="89">
         <v>6</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="62" t="s">
+      <c r="C10" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="62" t="s">
-        <v>98</v>
-      </c>
-      <c r="E10" s="47">
+      <c r="D10" s="57" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10" s="46">
         <v>99619.343603999994</v>
       </c>
-      <c r="F10" s="120"/>
-      <c r="G10" s="47">
+      <c r="F10" s="106"/>
+      <c r="G10" s="46">
         <f t="shared" si="1"/>
         <v>99619.343603999994</v>
       </c>
-      <c r="H10" s="47">
+      <c r="H10" s="46">
         <f t="shared" si="2"/>
         <v>4980.9671802000003</v>
       </c>
-      <c r="I10" s="109">
+      <c r="I10" s="95">
         <v>0.13200000000000001</v>
       </c>
-      <c r="J10" s="98"/>
-      <c r="K10" s="110">
+      <c r="J10" s="84"/>
+      <c r="K10" s="96">
         <f>E1*I10</f>
         <v>52361.048520000004</v>
       </c>
-      <c r="L10" s="110">
+      <c r="L10" s="96">
         <f t="shared" si="3"/>
         <v>156961.35930419998</v>
       </c>
-      <c r="M10" s="111">
+      <c r="M10" s="97">
         <f t="shared" si="4"/>
         <v>163239.81367636798</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="103">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" s="89">
         <v>7</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="62" t="s">
+      <c r="C11" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="62" t="s">
-        <v>62</v>
-      </c>
-      <c r="E11" s="47">
+      <c r="D11" s="57" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="46">
         <v>50377.675470000002</v>
       </c>
-      <c r="F11" s="120">
+      <c r="F11" s="106">
         <f t="shared" si="0"/>
         <v>50377.675470000002</v>
       </c>
-      <c r="G11" s="47">
+      <c r="G11" s="46">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H11" s="47">
+      <c r="H11" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I11" s="109">
+      <c r="I11" s="95">
         <v>0.127</v>
       </c>
-      <c r="J11" s="98"/>
-      <c r="K11" s="110">
+      <c r="J11" s="84"/>
+      <c r="K11" s="96">
         <f>E1*I11</f>
         <v>50377.675470000002</v>
       </c>
-      <c r="L11" s="110">
+      <c r="L11" s="96">
         <f t="shared" si="3"/>
         <v>50377.675470000002</v>
       </c>
-      <c r="M11" s="111">
+      <c r="M11" s="97">
         <f t="shared" si="4"/>
         <v>52392.782488800003</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="103">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" s="89">
         <v>8</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="62" t="s">
+      <c r="C12" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="62" t="s">
-        <v>61</v>
-      </c>
-      <c r="E12" s="47">
+      <c r="D12" s="57" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="46">
         <v>50377.675470000002</v>
       </c>
-      <c r="F12" s="120">
+      <c r="F12" s="106">
         <f>E12</f>
         <v>50377.675470000002</v>
       </c>
-      <c r="G12" s="47">
+      <c r="G12" s="46">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H12" s="47">
+      <c r="H12" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I12" s="109">
+      <c r="I12" s="95">
         <v>0.127</v>
       </c>
-      <c r="J12" s="98"/>
-      <c r="K12" s="110">
+      <c r="J12" s="84"/>
+      <c r="K12" s="96">
         <f>E1*I12</f>
         <v>50377.675470000002</v>
       </c>
-      <c r="L12" s="110">
+      <c r="L12" s="96">
         <f t="shared" si="3"/>
         <v>50377.675470000002</v>
       </c>
-      <c r="M12" s="111">
+      <c r="M12" s="97">
         <f t="shared" si="4"/>
         <v>52392.782488800003</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="112" t="s">
+    <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="113"/>
-      <c r="C13" s="114"/>
-      <c r="D13" s="114"/>
-      <c r="E13" s="115">
+      <c r="B13" s="99"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="101">
         <f>SUM(E5:E12)</f>
         <v>443932.90508400003</v>
       </c>
-      <c r="F13" s="104">
+      <c r="F13" s="90">
         <f>SUM(F5:F12)</f>
         <v>360987.84211000003</v>
       </c>
-      <c r="G13" s="104"/>
-      <c r="H13" s="104">
+      <c r="G13" s="90"/>
+      <c r="H13" s="90">
         <f>SUM(H5:H12)</f>
         <v>4980.9671802000003</v>
       </c>
-      <c r="I13" s="105">
+      <c r="I13" s="91">
         <f t="shared" ref="I13" si="5">SUM(I5:I12)</f>
         <v>1</v>
       </c>
-      <c r="J13" s="105">
+      <c r="J13" s="91">
         <f>SUM(J5:J12)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="115">
+      <c r="K13" s="101">
         <f>SUM(K5:K12)</f>
         <v>396674.61000000004</v>
       </c>
-      <c r="L13" s="115">
+      <c r="L13" s="101">
         <f>SUM(L5:L12)</f>
         <v>484600.64015420002</v>
       </c>
-      <c r="M13" s="116">
+      <c r="M13" s="102">
         <f>SUM(M5:M12)</f>
         <v>503984.66576036799</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="55" t="s">
+    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="53" t="s">
         <v>53</v>
       </c>
       <c r="E16">
         <v>7454</v>
       </c>
     </row>
-    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
-      <c r="D17" s="74"/>
+      <c r="D17" s="62"/>
       <c r="E17">
         <v>14805</v>
       </c>
@@ -2483,12 +2488,12 @@
       <c r="G17" s="29"/>
       <c r="H17" s="29"/>
       <c r="I17" s="29"/>
-      <c r="J17" s="56"/>
-      <c r="K17" s="56"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="32"/>
-    </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+      <c r="J17" s="54"/>
+      <c r="K17" s="54"/>
+      <c r="L17" s="54"/>
+      <c r="M17" s="31"/>
+    </row>
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>0</v>
       </c>
@@ -2513,15 +2518,15 @@
         <v>6</v>
       </c>
       <c r="J18" s="1"/>
-      <c r="K18" s="57" t="s">
+      <c r="K18" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="L18" s="46"/>
-      <c r="M18" s="46" t="s">
+      <c r="L18" s="45"/>
+      <c r="M18" s="45" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -2533,22 +2538,22 @@
         <v>49</v>
       </c>
       <c r="G19" s="2"/>
-      <c r="H19" s="38">
+      <c r="H19" s="37">
         <v>0.02</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>7</v>
       </c>
       <c r="J19" s="1"/>
-      <c r="K19" s="44" t="s">
+      <c r="K19" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="L19" s="39"/>
-      <c r="M19" s="39" t="s">
+      <c r="L19" s="38"/>
+      <c r="M19" s="38" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>1</v>
       </c>
@@ -2558,32 +2563,32 @@
       <c r="C20" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="75"/>
+      <c r="D20" s="63"/>
       <c r="E20">
         <v>3056</v>
       </c>
-      <c r="F20" s="47">
+      <c r="F20" s="46">
         <v>37971</v>
       </c>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52">
+      <c r="G20" s="50"/>
+      <c r="H20" s="50">
         <v>0</v>
       </c>
       <c r="I20" s="17">
         <v>0.121</v>
       </c>
-      <c r="J20" s="96"/>
-      <c r="K20" s="45">
+      <c r="J20" s="82"/>
+      <c r="K20" s="44">
         <f>0*I20</f>
         <v>0</v>
       </c>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42" t="e">
+      <c r="L20" s="41"/>
+      <c r="M20" s="41" t="e">
         <f>+#REF!+H20+K20</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>2</v>
       </c>
@@ -2593,32 +2598,32 @@
       <c r="C21" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="75"/>
+      <c r="D21" s="63"/>
       <c r="E21">
         <v>3056</v>
       </c>
-      <c r="F21" s="47">
+      <c r="F21" s="46">
         <v>66612</v>
       </c>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52">
+      <c r="G21" s="50"/>
+      <c r="H21" s="50">
         <v>0</v>
       </c>
       <c r="I21" s="17">
         <v>0.122</v>
       </c>
-      <c r="J21" s="96"/>
-      <c r="K21" s="45">
+      <c r="J21" s="82"/>
+      <c r="K21" s="44">
         <f t="shared" ref="K21:K27" si="6">0*I21</f>
         <v>0</v>
       </c>
-      <c r="L21" s="42"/>
-      <c r="M21" s="42" t="e">
+      <c r="L21" s="41"/>
+      <c r="M21" s="41" t="e">
         <f>+#REF!+H21+K21</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>3</v>
       </c>
@@ -2628,33 +2633,33 @@
       <c r="C22" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="75"/>
+      <c r="D22" s="63"/>
       <c r="E22">
         <f>SUM(E14:E21)</f>
         <v>34845</v>
       </c>
-      <c r="F22" s="47">
-        <v>0</v>
-      </c>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52">
+      <c r="F22" s="46">
+        <v>0</v>
+      </c>
+      <c r="G22" s="50"/>
+      <c r="H22" s="50">
         <v>0</v>
       </c>
       <c r="I22" s="17">
         <v>0.11700000000000001</v>
       </c>
-      <c r="J22" s="96"/>
-      <c r="K22" s="45">
+      <c r="J22" s="82"/>
+      <c r="K22" s="44">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L22" s="42"/>
-      <c r="M22" s="42" t="e">
+      <c r="L22" s="41"/>
+      <c r="M22" s="41" t="e">
         <f>+#REF!+H22+K22</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>4</v>
       </c>
@@ -2664,29 +2669,29 @@
       <c r="C23" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="75"/>
-      <c r="F23" s="47">
-        <v>0</v>
-      </c>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52">
+      <c r="D23" s="63"/>
+      <c r="F23" s="46">
+        <v>0</v>
+      </c>
+      <c r="G23" s="50"/>
+      <c r="H23" s="50">
         <v>0</v>
       </c>
       <c r="I23" s="17">
         <v>0.11700000000000001</v>
       </c>
-      <c r="J23" s="96"/>
-      <c r="K23" s="45">
+      <c r="J23" s="82"/>
+      <c r="K23" s="44">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L23" s="42"/>
-      <c r="M23" s="42" t="e">
+      <c r="L23" s="41"/>
+      <c r="M23" s="41" t="e">
         <f>+#REF!+H23+K23</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>5</v>
       </c>
@@ -2696,29 +2701,29 @@
       <c r="C24" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="75"/>
-      <c r="F24" s="47">
+      <c r="D24" s="63"/>
+      <c r="F24" s="46">
         <v>80517</v>
       </c>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52">
+      <c r="G24" s="50"/>
+      <c r="H24" s="50">
         <v>0</v>
       </c>
       <c r="I24" s="17">
         <v>0.13700000000000001</v>
       </c>
-      <c r="J24" s="96"/>
-      <c r="K24" s="45">
+      <c r="J24" s="82"/>
+      <c r="K24" s="44">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L24" s="42"/>
-      <c r="M24" s="42" t="e">
+      <c r="L24" s="41"/>
+      <c r="M24" s="41" t="e">
         <f>+#REF!+H24+K24</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>6</v>
       </c>
@@ -2728,29 +2733,29 @@
       <c r="C25" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D25" s="75"/>
-      <c r="F25" s="47">
-        <v>0</v>
-      </c>
-      <c r="G25" s="52"/>
-      <c r="H25" s="52">
+      <c r="D25" s="63"/>
+      <c r="F25" s="46">
+        <v>0</v>
+      </c>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50">
         <v>0</v>
       </c>
       <c r="I25" s="17">
         <v>0.13200000000000001</v>
       </c>
-      <c r="J25" s="96"/>
-      <c r="K25" s="45">
+      <c r="J25" s="82"/>
+      <c r="K25" s="44">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L25" s="42"/>
-      <c r="M25" s="42" t="e">
+      <c r="L25" s="41"/>
+      <c r="M25" s="41" t="e">
         <f>+#REF!+H25+K25</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>7</v>
       </c>
@@ -2760,32 +2765,32 @@
       <c r="C26" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="75"/>
+      <c r="D26" s="63"/>
       <c r="E26" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="47">
+      <c r="F26" s="46">
         <v>18542</v>
       </c>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52">
+      <c r="G26" s="50"/>
+      <c r="H26" s="50">
         <v>0</v>
       </c>
       <c r="I26" s="17">
         <v>0.127</v>
       </c>
-      <c r="J26" s="96"/>
-      <c r="K26" s="45">
+      <c r="J26" s="82"/>
+      <c r="K26" s="44">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L26" s="42"/>
-      <c r="M26" s="42" t="e">
+      <c r="L26" s="41"/>
+      <c r="M26" s="41" t="e">
         <f>+#REF!+H26+K26</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>8</v>
       </c>
@@ -2795,47 +2800,47 @@
       <c r="C27" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="D27" s="75"/>
+      <c r="D27" s="63"/>
       <c r="E27" t="s">
         <v>19</v>
       </c>
-      <c r="F27" s="47">
-        <v>0</v>
-      </c>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52">
+      <c r="F27" s="46">
+        <v>0</v>
+      </c>
+      <c r="G27" s="50"/>
+      <c r="H27" s="50">
         <v>0</v>
       </c>
       <c r="I27" s="17">
         <v>0.127</v>
       </c>
-      <c r="J27" s="96"/>
-      <c r="K27" s="45">
+      <c r="J27" s="82"/>
+      <c r="K27" s="44">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L27" s="42"/>
-      <c r="M27" s="42" t="e">
+      <c r="L27" s="41"/>
+      <c r="M27" s="41" t="e">
         <f>+#REF!+H27+K27</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="10"/>
-      <c r="D28" s="73"/>
+      <c r="D28" s="61"/>
       <c r="E28" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="50">
+      <c r="F28" s="48">
         <f>SUM(F20:F27)</f>
         <v>203642</v>
       </c>
-      <c r="G28" s="50"/>
-      <c r="H28" s="53">
+      <c r="G28" s="48"/>
+      <c r="H28" s="51">
         <f>SUM(H20:H27)</f>
         <v>0</v>
       </c>
@@ -2843,27 +2848,27 @@
         <f t="shared" ref="I28:K28" si="7">SUM(I20:I27)</f>
         <v>1</v>
       </c>
-      <c r="J28" s="97"/>
-      <c r="K28" s="40">
+      <c r="J28" s="83"/>
+      <c r="K28" s="39">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43" t="e">
+      <c r="L28" s="42"/>
+      <c r="M28" s="42" t="e">
         <f>SUM(M20:M27)</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="I30" s="60"/>
-      <c r="J30" s="60"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="I31" s="60"/>
-      <c r="J31" s="60"/>
-    </row>
-    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E39" s="54"/>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I30" s="56"/>
+      <c r="J30" s="56"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I31" s="56"/>
+      <c r="J31" s="56"/>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E39" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2889,574 +2894,439 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" customWidth="1"/>
-    <col min="9" max="9" width="0.140625" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="0.140625" customWidth="1"/>
-    <col min="12" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="13" customWidth="1"/>
+    <col min="1" max="1" width="6.21875" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.21875" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="D1" s="58">
-        <v>50000</v>
-      </c>
-      <c r="H1" s="137">
-        <v>250000</v>
-      </c>
-      <c r="I1" s="137"/>
-      <c r="J1" s="137"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="129" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="P2" s="21"/>
-    </row>
-    <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="31" t="s">
+      <c r="B1" s="130"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="132">
+        <v>108000</v>
+      </c>
+      <c r="E1" s="132"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="133"/>
+      <c r="L1" s="21"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="134" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="125"/>
+      <c r="C2" s="126"/>
+      <c r="D2" s="76" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="29"/>
-      <c r="F3" s="31" t="s">
+      <c r="E2" s="125"/>
+      <c r="F2" s="76" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="32"/>
-      <c r="P3" s="21"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="125"/>
+      <c r="J2" s="135"/>
+      <c r="L2" s="21"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="139" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C3" s="113" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="D3" s="122" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="121" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="122" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="122" t="s">
+        <v>96</v>
+      </c>
+      <c r="H3" s="121" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="127" t="s">
+        <v>95</v>
+      </c>
+      <c r="J3" s="136" t="s">
+        <v>58</v>
+      </c>
+      <c r="L3" s="21"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="140"/>
+      <c r="B4" s="114"/>
+      <c r="C4" s="114"/>
+      <c r="D4" s="122"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="122"/>
+      <c r="G4" s="122"/>
+      <c r="H4" s="121"/>
+      <c r="I4" s="127"/>
+      <c r="J4" s="136"/>
+      <c r="L4" s="21"/>
+    </row>
+    <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="138">
+        <v>1</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="124" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="96">
+        <v>0</v>
+      </c>
+      <c r="E5" s="96">
+        <v>0</v>
+      </c>
+      <c r="F5" s="96">
+        <v>42383</v>
+      </c>
+      <c r="G5" s="128">
+        <f>F5*1.48</f>
+        <v>62726.84</v>
+      </c>
+      <c r="H5" s="95">
+        <v>0.121</v>
+      </c>
+      <c r="I5" s="96">
+        <f>D$1*H5</f>
+        <v>13068</v>
+      </c>
+      <c r="J5" s="137">
+        <f>+F5+G5+I5</f>
+        <v>118177.84</v>
+      </c>
+      <c r="L5" s="21"/>
+    </row>
+    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="138">
+        <v>2</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="124" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="96">
+        <v>0</v>
+      </c>
+      <c r="E6" s="96">
+        <v>0</v>
+      </c>
+      <c r="F6" s="96">
+        <v>54967</v>
+      </c>
+      <c r="G6" s="128">
+        <f t="shared" ref="G6:G12" si="0">F6*1.48</f>
+        <v>81351.16</v>
+      </c>
+      <c r="H6" s="95">
+        <v>0.122</v>
+      </c>
+      <c r="I6" s="96">
+        <f t="shared" ref="I6:I12" si="1">D$1*H6</f>
+        <v>13176</v>
+      </c>
+      <c r="J6" s="137">
+        <f t="shared" ref="J6:J12" si="2">+F6+G6+I6</f>
+        <v>149494.16</v>
+      </c>
+      <c r="L6" s="21"/>
+    </row>
+    <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="138">
+        <v>3</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="124" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="96">
+        <v>0</v>
+      </c>
+      <c r="E7" s="96">
+        <v>0</v>
+      </c>
+      <c r="F7" s="96">
+        <v>0</v>
+      </c>
+      <c r="G7" s="128">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H7" s="95">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="I7" s="96">
+        <f t="shared" si="1"/>
+        <v>12636</v>
+      </c>
+      <c r="J7" s="137">
+        <f t="shared" si="2"/>
+        <v>12636</v>
+      </c>
+      <c r="L7" s="21"/>
+    </row>
+    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="138">
+        <v>4</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="124" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="96">
+        <v>0</v>
+      </c>
+      <c r="E8" s="96">
+        <v>0</v>
+      </c>
+      <c r="F8" s="96">
+        <v>52714</v>
+      </c>
+      <c r="G8" s="128">
+        <f t="shared" si="0"/>
+        <v>78016.72</v>
+      </c>
+      <c r="H8" s="95">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="I8" s="96">
+        <f t="shared" si="1"/>
+        <v>12636</v>
+      </c>
+      <c r="J8" s="137">
+        <f t="shared" si="2"/>
+        <v>143366.72</v>
+      </c>
+      <c r="L8" s="21"/>
+    </row>
+    <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="138">
+        <v>5</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="124" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="96">
+        <v>0</v>
+      </c>
+      <c r="E9" s="96">
+        <v>0</v>
+      </c>
+      <c r="F9" s="96">
+        <v>47988</v>
+      </c>
+      <c r="G9" s="128">
+        <f t="shared" si="0"/>
+        <v>71022.240000000005</v>
+      </c>
+      <c r="H9" s="95">
+        <v>0.13700000000000001</v>
+      </c>
+      <c r="I9" s="96">
+        <f t="shared" si="1"/>
+        <v>14796.000000000002</v>
+      </c>
+      <c r="J9" s="137">
+        <f t="shared" si="2"/>
+        <v>133806.24000000002</v>
+      </c>
+      <c r="L9" s="21"/>
+    </row>
+    <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="138">
         <v>6</v>
       </c>
-      <c r="I4" s="57" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="K4" s="71"/>
-      <c r="L4" s="135" t="s">
-        <v>72</v>
-      </c>
-      <c r="M4" s="81" t="s">
-        <v>5</v>
-      </c>
-      <c r="N4" s="133" t="s">
-        <v>59</v>
-      </c>
-      <c r="P4" s="21"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="38">
-        <v>0.02</v>
-      </c>
-      <c r="H5" s="2" t="s">
+      <c r="B10" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="124" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="96">
+        <v>0</v>
+      </c>
+      <c r="E10" s="96">
+        <v>0</v>
+      </c>
+      <c r="F10" s="96">
+        <v>46236</v>
+      </c>
+      <c r="G10" s="128">
+        <f t="shared" si="0"/>
+        <v>68429.279999999999</v>
+      </c>
+      <c r="H10" s="95">
+        <v>0.13200000000000001</v>
+      </c>
+      <c r="I10" s="96">
+        <f t="shared" si="1"/>
+        <v>14256</v>
+      </c>
+      <c r="J10" s="137">
+        <f t="shared" si="2"/>
+        <v>128921.28</v>
+      </c>
+      <c r="L10" s="21"/>
+    </row>
+    <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="138">
         <v>7</v>
       </c>
-      <c r="I5" s="44" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5" s="68" t="s">
-        <v>71</v>
-      </c>
-      <c r="K5" s="61"/>
-      <c r="L5" s="136"/>
-      <c r="M5" s="82" t="s">
-        <v>73</v>
-      </c>
-      <c r="N5" s="134"/>
-      <c r="P5" s="21"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+      <c r="B11" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="124" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="96">
+        <v>0</v>
+      </c>
+      <c r="E11" s="96">
+        <v>0</v>
+      </c>
+      <c r="F11" s="96">
+        <v>0</v>
+      </c>
+      <c r="G11" s="128">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="95">
+        <v>0.127</v>
+      </c>
+      <c r="I11" s="96">
+        <f t="shared" si="1"/>
+        <v>13716</v>
+      </c>
+      <c r="J11" s="137">
+        <f t="shared" si="2"/>
+        <v>13716</v>
+      </c>
+      <c r="L11" s="21"/>
+    </row>
+    <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="138">
+        <v>8</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="124" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="96">
+        <v>0</v>
+      </c>
+      <c r="E12" s="96">
+        <v>0</v>
+      </c>
+      <c r="F12" s="96">
+        <v>0</v>
+      </c>
+      <c r="G12" s="128">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="95">
+        <v>0.127</v>
+      </c>
+      <c r="I12" s="96">
+        <f t="shared" si="1"/>
+        <v>13716</v>
+      </c>
+      <c r="J12" s="137">
+        <f t="shared" si="2"/>
+        <v>13716</v>
+      </c>
+      <c r="L12" s="21"/>
+    </row>
+    <row r="13" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="98" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="99"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="101">
+        <f>SUM(D5:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="101">
+        <f>SUM(E5:E12)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="101">
+        <f t="shared" ref="F13" si="3">SUM(F5:F12)</f>
+        <v>244288</v>
+      </c>
+      <c r="G13" s="101">
+        <f>SUM(G5:G12)</f>
+        <v>361546.23999999999</v>
+      </c>
+      <c r="H13" s="91">
+        <f t="shared" ref="H13" si="4">SUM(H5:H12)</f>
         <v>1</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="63" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="47">
-        <v>0</v>
-      </c>
-      <c r="E6" s="47">
-        <v>0</v>
-      </c>
-      <c r="F6" s="47">
-        <f>+D6-E6</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="52">
-        <v>0</v>
-      </c>
-      <c r="H6" s="17">
-        <v>0.121</v>
-      </c>
-      <c r="I6" s="45">
-        <f>H$1*H6</f>
-        <v>30250</v>
-      </c>
-      <c r="J6" s="69">
-        <v>9706.619999999999</v>
-      </c>
-      <c r="K6" s="72"/>
-      <c r="L6" s="69">
-        <f>(J6+K6)*5%+(J6+K6)*5%+(J6+K6)*5%+(J6+K6)*5%+(J6+K6)*5%</f>
-        <v>2426.6549999999997</v>
-      </c>
-      <c r="M6" s="47">
-        <f>H$1*H6</f>
-        <v>30250</v>
-      </c>
-      <c r="N6" s="70">
-        <f>J6+K6+L6+M6</f>
-        <v>42383.274999999994</v>
-      </c>
-      <c r="P6" s="21"/>
-    </row>
-    <row r="7" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
-        <v>2</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="63" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="47">
-        <v>0</v>
-      </c>
-      <c r="E7" s="47">
-        <v>0</v>
-      </c>
-      <c r="F7" s="47">
-        <f t="shared" ref="F7:F13" si="0">+D7-E7</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="52">
-        <v>0</v>
-      </c>
-      <c r="H7" s="17">
-        <v>0.122</v>
-      </c>
-      <c r="I7" s="45">
-        <f t="shared" ref="I7:I13" si="1">H$1*H7</f>
-        <v>30500</v>
-      </c>
-      <c r="J7" s="69">
-        <v>19573.68</v>
-      </c>
-      <c r="K7" s="72"/>
-      <c r="L7" s="69">
-        <f t="shared" ref="L7:L13" si="2">(J7+K7)*5%+(J7+K7)*5%+(J7+K7)*5%+(J7+K7)*5%+(J7+K7)*5%</f>
-        <v>4893.42</v>
-      </c>
-      <c r="M7" s="47">
-        <f t="shared" ref="M7:M13" si="3">H$1*H7</f>
-        <v>30500</v>
-      </c>
-      <c r="N7" s="70">
-        <f t="shared" ref="N7:N13" si="4">J7+K7+L7+M7</f>
-        <v>54967.1</v>
-      </c>
-      <c r="P7" s="21"/>
-    </row>
-    <row r="8" spans="1:16" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
-        <v>3</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="63" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="47">
-        <v>0</v>
-      </c>
-      <c r="E8" s="47">
-        <v>0</v>
-      </c>
-      <c r="F8" s="47">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="52">
-        <v>0</v>
-      </c>
-      <c r="H8" s="17">
-        <v>0.11700000000000001</v>
-      </c>
-      <c r="I8" s="45">
-        <f t="shared" si="1"/>
-        <v>29250</v>
-      </c>
-      <c r="J8" s="69">
-        <v>0</v>
-      </c>
-      <c r="K8" s="72"/>
-      <c r="L8" s="69">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M8" s="47">
-        <f t="shared" si="3"/>
-        <v>29250</v>
-      </c>
-      <c r="N8" s="70">
-        <f t="shared" si="4"/>
-        <v>29250</v>
-      </c>
-      <c r="P8" s="21"/>
-    </row>
-    <row r="9" spans="1:16" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A9" s="11">
-        <v>4</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="63" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="47">
-        <v>0</v>
-      </c>
-      <c r="E9" s="47">
-        <v>0</v>
-      </c>
-      <c r="F9" s="47">
-        <f>+D9-E9</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="52">
-        <v>0</v>
-      </c>
-      <c r="H9" s="17">
-        <v>0.11700000000000001</v>
-      </c>
-      <c r="I9" s="45">
-        <f t="shared" si="1"/>
-        <v>29250</v>
-      </c>
-      <c r="J9" s="69">
-        <v>18771.480000000003</v>
-      </c>
-      <c r="K9" s="72"/>
-      <c r="L9" s="69">
-        <f t="shared" si="2"/>
-        <v>4692.8700000000008</v>
-      </c>
-      <c r="M9" s="47">
-        <f t="shared" si="3"/>
-        <v>29250</v>
-      </c>
-      <c r="N9" s="70">
-        <f t="shared" si="4"/>
-        <v>52714.350000000006</v>
-      </c>
-      <c r="P9" s="21"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
-        <v>5</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="63" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="47">
-        <v>0</v>
-      </c>
-      <c r="E10" s="47">
-        <v>0</v>
-      </c>
-      <c r="F10" s="47">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="52">
-        <v>0</v>
-      </c>
-      <c r="H10" s="17">
-        <v>0.13700000000000001</v>
-      </c>
-      <c r="I10" s="45">
-        <f t="shared" si="1"/>
-        <v>34250</v>
-      </c>
-      <c r="J10" s="69">
-        <v>10990.140000000001</v>
-      </c>
-      <c r="K10" s="72"/>
-      <c r="L10" s="69">
-        <f t="shared" si="2"/>
-        <v>2747.5350000000003</v>
-      </c>
-      <c r="M10" s="47">
-        <f t="shared" si="3"/>
-        <v>34250</v>
-      </c>
-      <c r="N10" s="70">
-        <f t="shared" si="4"/>
-        <v>47987.675000000003</v>
-      </c>
-      <c r="P10" s="21"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="11">
-        <v>6</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="63" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="47">
-        <v>0</v>
-      </c>
-      <c r="E11" s="47">
-        <v>0</v>
-      </c>
-      <c r="F11" s="47">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="52">
-        <v>0</v>
-      </c>
-      <c r="H11" s="17">
-        <v>0.13200000000000001</v>
-      </c>
-      <c r="I11" s="45">
-        <f t="shared" si="1"/>
-        <v>33000</v>
-      </c>
-      <c r="J11" s="69">
-        <v>10589.04</v>
-      </c>
-      <c r="K11" s="72"/>
-      <c r="L11" s="69">
-        <f t="shared" si="2"/>
-        <v>2647.2600000000007</v>
-      </c>
-      <c r="M11" s="47">
-        <f t="shared" si="3"/>
-        <v>33000</v>
-      </c>
-      <c r="N11" s="70">
-        <f t="shared" si="4"/>
-        <v>46236.3</v>
-      </c>
-      <c r="P11" s="21"/>
-    </row>
-    <row r="12" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
-        <v>7</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="63" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="47">
-        <v>0</v>
-      </c>
-      <c r="E12" s="47">
-        <v>0</v>
-      </c>
-      <c r="F12" s="47">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="52">
-        <v>0</v>
-      </c>
-      <c r="H12" s="17">
-        <v>0.127</v>
-      </c>
-      <c r="I12" s="45">
-        <f t="shared" si="1"/>
-        <v>31750</v>
-      </c>
-      <c r="J12" s="69">
-        <v>0</v>
-      </c>
-      <c r="K12" s="72"/>
-      <c r="L12" s="69">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M12" s="47">
-        <f t="shared" si="3"/>
-        <v>31750</v>
-      </c>
-      <c r="N12" s="70">
-        <f t="shared" si="4"/>
-        <v>31750</v>
-      </c>
-      <c r="P12" s="21"/>
-    </row>
-    <row r="13" spans="1:16" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A13" s="11">
-        <v>8</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="63" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" s="47">
-        <v>0</v>
-      </c>
-      <c r="E13" s="47">
-        <v>0</v>
-      </c>
-      <c r="F13" s="47">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="52">
-        <v>0</v>
-      </c>
-      <c r="H13" s="17">
-        <v>0.127</v>
-      </c>
-      <c r="I13" s="45">
-        <f t="shared" si="1"/>
-        <v>31750</v>
-      </c>
-      <c r="J13" s="69">
-        <v>0</v>
-      </c>
-      <c r="K13" s="72"/>
-      <c r="L13" s="69">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M13" s="47">
-        <f t="shared" si="3"/>
-        <v>31750</v>
-      </c>
-      <c r="N13" s="70">
-        <f t="shared" si="4"/>
-        <v>31750</v>
-      </c>
-      <c r="P13" s="21"/>
-    </row>
-    <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="48">
-        <f>SUM(D6:D13)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="50">
-        <f>SUM(E6:E13)</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="48">
-        <f t="shared" ref="F14" si="5">SUM(F6:F13)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="53">
-        <f>SUM(G6:G13)</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="15">
-        <f t="shared" ref="H14:I14" si="6">SUM(H6:H13)</f>
-        <v>1</v>
-      </c>
-      <c r="I14" s="40">
-        <f t="shared" si="6"/>
-        <v>250000</v>
-      </c>
-      <c r="J14" s="43">
-        <f>SUM(J6:J13)</f>
-        <v>69630.959999999992</v>
-      </c>
-      <c r="K14" s="43">
-        <f>SUM(K6:K13)</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43">
-        <f>SUM(M6:M13)</f>
-        <v>250000</v>
-      </c>
-      <c r="N14" s="40">
-        <f>SUM(N6:N13)</f>
-        <v>337038.7</v>
-      </c>
-      <c r="P14" s="21"/>
+      <c r="I13" s="101">
+        <f>SUM(I5:I12)</f>
+        <v>108000</v>
+      </c>
+      <c r="J13" s="102">
+        <f>SUM(J5:J12)</f>
+        <v>713834.24</v>
+      </c>
+      <c r="L13" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="H1:J1"/>
+  <mergeCells count="11">
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="85" orientation="portrait" r:id="rId1"/>

</xml_diff>